<commit_message>
feat: initialize comprehensive SISTEKIN 2026 OBE curriculum documentation and management tools
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/006_DISTRIBUSI_DAN_PANDUAN_MK_PEMINATAN_MBKM.xlsx
+++ b/KURIKULUM2026_REVISI/006_DISTRIBUSI_DAN_PANDUAN_MK_PEMINATAN_MBKM.xlsx
@@ -496,7 +496,7 @@
   <cols>
     <col width="69" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="33.34999999999999" customWidth="1" min="3" max="3"/>
+    <col width="36.8" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -609,7 +609,7 @@
       <c r="B9" s="7" t="inlineStr"/>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>• STI-519 Keamanan Lanjut (3)</t>
+          <t>• STI-626 Deep Learning (+P) (3)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>

</xml_diff>